<commit_message>
F9 (preparación): TP1–TP6 a ronghe RH-5016 (Keystone 5016 en 0 en LCSC), conteo del formulario (118 SMD, 8 THT, 2 BGA/QFP), guía con cada campo de PCBWay, DigiKey con K1 y repuestos (US$ 17,87, cupo US$ 40)
</commit_message>
<xml_diff>
--- a/docs/fabricacion/BOM_PCBWay.xlsx
+++ b/docs/fabricacion/BOM_PCBWay.xlsx
@@ -1646,7 +1646,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -3228,12 +3228,12 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Keystone Electronics</t>
+          <t>ronghe</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>5016</t>
+          <t>RH-5016</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -3263,10 +3263,14 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>LCSC C238129</t>
-        </is>
-      </c>
-      <c r="L51" s="2" t="inlineStr"/>
+          <t>LCSC C5199799</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>cambio (22 oct): el Keystone 5016 está en 0 en LCSC; el RH-5016 es el mismo plano (3,81 × 2,84 mm)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">

</xml_diff>

<commit_message>
F9 (preparación): sin DigiKey (D19). K1 AQY414EHAX lo compra y lo suelda PCBWay (DigiKey/Mouser) y F1/F2 llevan 2 fusibles 3403.0274.11 de repuesto; BOM, Pick & Place (127 piezas), notas (597 caracteres), parámetros de Altium y carrito actualizados
</commit_message>
<xml_diff>
--- a/docs/fabricacion/BOM_PCBWay.xlsx
+++ b/docs/fabricacion/BOM_PCBWay.xlsx
@@ -1496,7 +1496,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>cambio: el mismo UMT-H T1A en bolsa; el .23 (carrete) está en 0 en LCSC</t>
+          <t>Please buy 2 extra pcs (4 total) and ship the 2 spares loose with the boards</t>
         </is>
       </c>
     </row>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -1916,22 +1916,22 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>Panasonic</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>LQH43NH120J03L</t>
+          <t>AQY414EHAX</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Inductor 12 uH 5% 420 mA 0.25 ohm 1812, AEC-Q200</t>
+          <t>PhotoMOS 1 Form B (NC), 400 V 120 mA, reinforced insulation 5000 Vrms, SMD DIP-4</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>RLS126</t>
+          <t>SOP254P962X315-4N</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1951,12 +1951,12 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>LCSC C3224514</t>
+          <t>DigiKey 255-6089-1-ND</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>cambio: RECOM RLS-126 sin stock en LCSC; 12 uH, 0,25 ohm, 420 mA, AEC-Q200</t>
+          <t>Not in LCSC stock: please buy from DigiKey 255-6089-1-ND or Mouser 769-AQY414EHAX. No substitutes</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -1974,22 +1974,22 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>Murata</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>SRR4028-2R2Y</t>
+          <t>LQH43NH120J03L</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Inductor</t>
+          <t>Inductor 12 uH 5% 420 mA 0.25 ohm 1812, AEC-Q200</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>SRR4028</t>
+          <t>RLS126</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2009,10 +2009,14 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>LCSC C2041777</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr"/>
+          <t>LCSC C3224514</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>cambio: RECOM RLS-126 sin stock en LCSC; 12 uH, 0,25 ohm, 420 mA, AEC-Q200</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -2020,30 +2024,30 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>LED1, LED2, LED3, LED4</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Kingbright</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>APT2012SGC</t>
+          <t>SRR4028-2R2Y</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>LED</t>
+          <t>Inductor</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>LEDC2012X85N</t>
+          <t>SRR4028</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2063,7 +2067,7 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>LCSC C5353439</t>
+          <t>LCSC C2041777</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr"/>
@@ -2074,11 +2078,11 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>LED5</t>
+          <t>LED1, LED2, LED3, LED4</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
@@ -2087,7 +2091,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>APT2012SURCK</t>
+          <t>APT2012SGC</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2117,7 +2121,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>LCSC C5875730</t>
+          <t>LCSC C5353439</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr"/>
@@ -2128,7 +2132,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>LED6</t>
+          <t>LED5</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2136,17 +2140,17 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Hubei KENTO Electronic</t>
+          <t>Kingbright</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>KT-0805Y</t>
+          <t>APT2012SURCK</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>LED yellow 0805, 590 nm</t>
+          <t>LED</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2171,7 +2175,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>LCSC C2296</t>
+          <t>LCSC C5875730</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr"/>
@@ -2182,7 +2186,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>PS1</t>
+          <t>LED6</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2190,27 +2194,27 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Mean Well</t>
+          <t>Hubei KENTO Electronic</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>IRM-20-12</t>
+          <t>KT-0805Y</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Power Supply</t>
+          <t>LED yellow 0805, 590 nm</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>IRM2012</t>
+          <t>LEDC2012X85N</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>THT</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -2225,14 +2229,10 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>LCSC C5278499</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>antes Sigma, 71.400 COP (THT)</t>
-        </is>
-      </c>
+          <t>LCSC C2296</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -2240,35 +2240,35 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Q1, Q2</t>
+          <t>PS1</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>onsemi</t>
+          <t>Mean Well</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>MMBT3904LT1G</t>
+          <t>IRM-20-12</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Transistor BJT NPN</t>
+          <t>Power Supply</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>SOT96P237X111-3N</t>
+          <t>IRM2012</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>THT</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2283,10 +2283,14 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>LCSC C81464</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr"/>
+          <t>LCSC C5278499</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>antes Sigma, 71.400 COP (THT)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -2294,25 +2298,25 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q1, Q2</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Alpha &amp; Omega Semiconductor</t>
+          <t>onsemi</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>AO3400A</t>
+          <t>MMBT3904LT1G</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>MOSFET N-channel 30V 5.7A, Rds(on) 48mR max at Vgs 2.5V, SOT-23</t>
+          <t>Transistor BJT NPN</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -2337,7 +2341,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>LCSC C20917</t>
+          <t>LCSC C81464</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr"/>
@@ -2348,30 +2352,30 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>R1, R8, R15, R17, R25, R26, R28, R29, R30, R31, R39, R41</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Alpha &amp; Omega Semiconductor</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>RC0805FR-071KL</t>
+          <t>AO3400A</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Resistor</t>
+          <t>MOSFET N-channel 30V 5.7A, Rds(on) 48mR max at Vgs 2.5V, SOT-23</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>RESC2012X60N</t>
+          <t>SOT96P237X111-3N</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2391,7 +2395,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>LCSC C95781</t>
+          <t>LCSC C20917</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr"/>
@@ -2402,20 +2406,20 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>R10, R14</t>
+          <t>R1, R8, R15, R17, R25, R26, R28, R29, R30, R31, R39, R41</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>ERA-6AEB133V</t>
+          <t>RC0805FR-071KL</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2445,7 +2449,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>LCSC C445658</t>
+          <t>LCSC C95781</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr"/>
@@ -2456,7 +2460,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>R11, R13</t>
+          <t>R10, R14</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2464,17 +2468,17 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Panasonic</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>RT0805BRD0710RL</t>
+          <t>ERA-6AEB133V</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Resistencia de pelicula delgada 10 ohm 0.1% 25 ppm 0805</t>
+          <t>Resistor</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -2499,14 +2503,10 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>LCSC C865142</t>
-        </is>
-      </c>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>cambio: ERA-6AHD100V en 0 en LCSC; 0,1 % y 25 ppm (mejor)</t>
-        </is>
-      </c>
+          <t>LCSC C445658</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2514,11 +2514,11 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>R16, R18, R22, R27, R34, R40</t>
+          <t>R11, R13</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
@@ -2527,12 +2527,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>RC0805FR-0710KL</t>
+          <t>RT0805BRD0710RL</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Resistor</t>
+          <t>Resistencia de pelicula delgada 10 ohm 0.1% 25 ppm 0805</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -2557,10 +2557,14 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>LCSC C84376</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr"/>
+          <t>LCSC C865142</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>cambio: ERA-6AHD100V en 0 en LCSC; 0,1 % y 25 ppm (mejor)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2568,11 +2572,11 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>R19, R20</t>
+          <t>R16, R18, R22, R27, R34, R40</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
@@ -2581,7 +2585,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>RC0805FR-0712KL</t>
+          <t>RC0805FR-0710KL</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2611,7 +2615,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>LCSC C114556</t>
+          <t>LCSC C84376</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr"/>
@@ -2622,20 +2626,20 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>R2, R3, R4, R5</t>
+          <t>R19, R20</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>ERJ-P08F1004V</t>
+          <t>RC0805FR-0712KL</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2645,7 +2649,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>ERJP08_(1206)</t>
+          <t>RESC2012X60N</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2665,7 +2669,7 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>LCSC C41369755</t>
+          <t>LCSC C114556</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr"/>
@@ -2676,7 +2680,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>R21, R32, R33, R35</t>
+          <t>R2, R3, R4, R5</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2684,12 +2688,12 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Panasonic</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>RC0805FR-074K7L</t>
+          <t>ERJ-P08F1004V</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2699,7 +2703,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>RESC2012X60N</t>
+          <t>ERJP08_(1206)</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2719,7 +2723,7 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>LCSC C60816</t>
+          <t>LCSC C41369755</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr"/>
@@ -2730,11 +2734,11 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>R23, R24</t>
+          <t>R21, R32, R33, R35</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
@@ -2743,7 +2747,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>RC0805FR-075K1L</t>
+          <t>RC0805FR-074K7L</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2773,7 +2777,7 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>LCSC C84375</t>
+          <t>LCSC C60816</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr"/>
@@ -2784,11 +2788,11 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>R36</t>
+          <t>R23, R24</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
@@ -2797,7 +2801,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>RC0805FR-07100RL</t>
+          <t>RC0805FR-075K1L</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2827,7 +2831,7 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>LCSC C105577</t>
+          <t>LCSC C84375</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr"/>
@@ -2838,7 +2842,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>R37</t>
+          <t>R36</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -2851,7 +2855,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>RC1206FR-0768RL</t>
+          <t>RC0805FR-07100RL</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2861,7 +2865,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>ERJP08_(1206)</t>
+          <t>RESC2012X60N</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2881,7 +2885,7 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>LCSC C137238</t>
+          <t>LCSC C105577</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr"/>
@@ -2892,7 +2896,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>R38</t>
+          <t>R37</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -2905,7 +2909,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>RC0805FR-07330RL</t>
+          <t>RC1206FR-0768RL</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2915,7 +2919,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>RESC2012X60N</t>
+          <t>ERJP08_(1206)</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2935,7 +2939,7 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>LCSC C105878</t>
+          <t>LCSC C137238</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr"/>
@@ -2946,7 +2950,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R38</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -2954,12 +2958,12 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>ERA-6AEB103V</t>
+          <t>RC0805FR-07330RL</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2989,7 +2993,7 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>LCSC C191101</t>
+          <t>LCSC C105878</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr"/>
@@ -3000,7 +3004,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R6</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3008,12 +3012,12 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Panasonic</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>RC0805FR-0747KL</t>
+          <t>ERA-6AEB103V</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -3043,7 +3047,7 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>LCSC C126351</t>
+          <t>LCSC C191101</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr"/>
@@ -3054,20 +3058,20 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>R9, R12</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>ERA-6AEB203V</t>
+          <t>RC0805FR-0747KL</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3097,7 +3101,7 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>LCSC C473304</t>
+          <t>LCSC C126351</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr"/>
@@ -3108,30 +3112,30 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>RV1</t>
+          <t>R9, R12</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Ruilon</t>
+          <t>Panasonic</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>RL4032P471KJ</t>
+          <t>ERA-6AEB203V</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Varistor SMD 300 VAC, 470 V, 2500 A (8/20 us), 30 J, 4032</t>
+          <t>Resistor</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>CU4032</t>
+          <t>RESC2012X60N</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -3151,14 +3155,10 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>LCSC C2935514</t>
-        </is>
-      </c>
-      <c r="L49" s="2" t="inlineStr">
-        <is>
-          <t>cambio: TDK B72660M0301K072 sin stock en LCSC; 300 VAC, 2500 A, 30 J, mismos pads</t>
-        </is>
-      </c>
+          <t>LCSC C473304</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -3166,7 +3166,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>SW1</t>
+          <t>RV1</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3174,22 +3174,22 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>XKB Connectivity</t>
+          <t>Ruilon</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>TS-1187A-B-A-B</t>
+          <t>RL4032P471KJ</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Tact switch 5.1 x 5.1 x 1.5 mm, 160 gf, 50 mA 12 VDC</t>
+          <t>Varistor SMD 300 VAC, 470 V, 2500 A (8/20 us), 30 J, 4032</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>TS1187ABAB</t>
+          <t>CU4032</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -3209,10 +3209,14 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>LCSC C318884</t>
-        </is>
-      </c>
-      <c r="L50" s="2" t="inlineStr"/>
+          <t>LCSC C2935514</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>cambio: TDK B72660M0301K072 sin stock en LCSC; 300 VAC, 2500 A, 30 J, mismos pads</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -3220,30 +3224,30 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>TP1, TP2, TP3, TP4, TP5, TP6</t>
+          <t>SW1</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>ronghe</t>
+          <t>XKB Connectivity</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>RH-5016</t>
+          <t>TS-1187A-B-A-B</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Test Point, 1-Pin SMT, RoHS, Tape and Reel</t>
+          <t>Tact switch 5.1 x 5.1 x 1.5 mm, 160 gf, 50 mA 12 VDC</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE-5016_V</t>
+          <t>TS1187ABAB</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -3263,14 +3267,10 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>LCSC C5199799</t>
-        </is>
-      </c>
-      <c r="L51" s="2" t="inlineStr">
-        <is>
-          <t>cambio (22 oct): el Keystone 5016 está en 0 en LCSC; el RH-5016 es el mismo plano (3,81 × 2,84 mm)</t>
-        </is>
-      </c>
+          <t>LCSC C318884</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -3278,30 +3278,30 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>TP1, TP2, TP3, TP4, TP5, TP6</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>ronghe</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>AMC3330DWER</t>
+          <t>RH-5016</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Amplificador aislado +-1 V con DC/DC integrado, aislamiento reforzado, SOIC-16 DWE (carrete)</t>
+          <t>Test Point, 1-Pin SMT, RoHS, Tape and Reel</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>SOIC127P1030X265-16N</t>
+          <t>KEYSTONE-5016_V</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3321,12 +3321,12 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>LCSC C2999368</t>
+          <t>LCSC C5199799</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>cambio de MPN: DWE (tubo) en 0; DWER es la misma pieza en carrete</t>
+          <t>cambio (22 oct): el Keystone 5016 está en 0 en LCSC; el RH-5016 es el mismo plano (3,81 × 2,84 mm)</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3336,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3344,22 +3344,22 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Microchip</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>ATM90E26-YU-R</t>
+          <t>AMC3330DWER</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Integrated Circuit</t>
+          <t>Amplificador aislado +-1 V con DC/DC integrado, aislamiento reforzado, SOIC-16 DWE (carrete)</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>SOP65P778X199-28N</t>
+          <t>SOIC127P1030X265-16N</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3379,10 +3379,14 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>LCSC C616398</t>
-        </is>
-      </c>
-      <c r="L53" s="2" t="inlineStr"/>
+          <t>LCSC C2999368</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>cambio de MPN: DWE (tubo) en 0; DWER es la misma pieza en carrete</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -3390,7 +3394,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>U4</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3398,12 +3402,12 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Espressif Systems</t>
+          <t>Microchip</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>ESP32-S3-WROOM-1-N16R2</t>
+          <t>ATM90E26-YU-R</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3413,7 +3417,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>ESP32S3WROOM1N16R2</t>
+          <t>SOP65P778X199-28N</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3433,14 +3437,10 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>LCSC C2913205</t>
-        </is>
-      </c>
-      <c r="L54" s="2" t="inlineStr">
-        <is>
-          <t>antes Mouser</t>
-        </is>
-      </c>
+          <t>LCSC C616398</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -3448,7 +3448,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>U5</t>
+          <t>U4</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3456,22 +3456,22 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>WCH</t>
+          <t>Espressif Systems</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>CH340C</t>
+          <t>ESP32-S3-WROOM-1-N16R2</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>USB to UART bridge</t>
+          <t>Integrated Circuit</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>SOIC127P600X175-16N</t>
+          <t>ESP32S3WROOM1N16R2</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3491,10 +3491,14 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>LCSC C84681</t>
-        </is>
-      </c>
-      <c r="L55" s="2" t="inlineStr"/>
+          <t>LCSC C2913205</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>antes Mouser</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -3502,7 +3506,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>U6</t>
+          <t>U5</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3510,22 +3514,22 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Aosong</t>
+          <t>WCH</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>AHT20</t>
+          <t>CH340C</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Integrated Circuit</t>
+          <t>USB to UART bridge</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>AHT20</t>
+          <t>SOIC127P600X175-16N</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3545,7 +3549,7 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>LCSC C2757850</t>
+          <t>LCSC C84681</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr"/>
@@ -3556,7 +3560,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>U7</t>
+          <t>U6</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3564,22 +3568,22 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Analog Devices</t>
+          <t>Aosong</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>DS3231SN#T&amp;R</t>
+          <t>AHT20</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>I2C RTC with integrated TCXO and crystal, VBAT, SO-16W</t>
+          <t>Integrated Circuit</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>SOIC127P1030X265-16N</t>
+          <t>AHT20</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3599,7 +3603,7 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>LCSC C9866</t>
+          <t>LCSC C2757850</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr"/>
@@ -3610,7 +3614,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Y1</t>
+          <t>U7</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3618,103 +3622,99 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
+          <t>Analog Devices</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>DS3231SN#T&amp;R</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>I2C RTC with integrated TCXO and crystal, VBAT, SO-16W</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>SOIC127P1030X265-16N</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>SMD</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>PCBWay</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>PCBWay</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>LCSC C9866</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
           <t>ECS</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>ECS-81.92-12-30Q-EN-TR</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>Crystal or Oscillator</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
         <is>
           <t>ECS81921230QENTR</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>SMD</t>
-        </is>
-      </c>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>PCBWay</t>
-        </is>
-      </c>
-      <c r="J58" s="2" t="inlineStr">
-        <is>
-          <t>PCBWay</t>
-        </is>
-      </c>
-      <c r="K58" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>SMD</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>PCBWay</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>PCBWay</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
         <is>
           <t>LCSC C2450755</t>
         </is>
       </c>
-      <c r="L58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="n">
-        <v>58</v>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>K1</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>Panasonic</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>AQY414EHAX</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>PhotoMOS 1 Form B (NC), 400 V 120 mA, reinforced insulation 5000 Vrms, SMD DIP-4</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>SOP254P962X315-4N</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr">
-        <is>
-          <t>SMD</t>
-        </is>
-      </c>
-      <c r="I59" s="3" t="inlineStr">
-        <is>
-          <t>A mano (no ensamblar)</t>
-        </is>
-      </c>
-      <c r="J59" s="3" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="K59" s="3" t="inlineStr">
-        <is>
-          <t>255-6089-1-ND</t>
-        </is>
-      </c>
-      <c r="L59" s="3" t="inlineStr">
-        <is>
-          <t>LCSC en 0, sin equivalente NC con aislamiento reforzado</t>
-        </is>
-      </c>
+      <c r="L59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n">

</xml_diff>